<commit_message>
Fjern bokomslaget fra forsiden og juster tidsplanen uke 40
Forfatterens egne endringer, gjort parallelt med oppdateringen av
installasjonsinstruksene:

- index.Rmd: fjernet figuren med Keller-bokomslaget fra pensumavsnittet.
  Avsnittet omtaler nå boken som et supplement, ikke hovedkilde.
- tidsplan-H26.xlsx: uke 40 mandag endret til "(ingen aktivitet - jobb
  med obligatorisk innlevering)", likt torsdagscellen samme uke.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/diverse/tidsplan-H26.xlsx
+++ b/diverse/tidsplan-H26.xlsx
@@ -1,12 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\met4\diverse\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BB54A47-2322-4A5B-B09F-6ADAC7A1507C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-28800" yWindow="1935" windowWidth="29010" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -18,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
   <si>
     <t>Uke</t>
   </si>
@@ -44,9 +51,6 @@
     <t>Mandag 10:15 - 12:00</t>
   </si>
   <si>
-    <t>17.08: **Introduksjon til MET4** . Aud A</t>
-  </si>
-  <si>
     <t>24.08: **Oversiktsforelesning Grunnleggende statistikk** i Aud A</t>
   </si>
   <si>
@@ -56,9 +60,6 @@
     <t>15.10: **Oppgaveseminar 5** Aud A. Se \@ref(seminar) for oppgaver.</t>
   </si>
   <si>
-    <t>29.10: **Oppgaveseminar  6**, Aud A. Se \@ref(seminar) for oppgaver.</t>
-  </si>
-  <si>
     <t>27.08: **Oppgaveseminar 1** i Aud A. Se \@ref(seminar) for oppgaver.</t>
   </si>
   <si>
@@ -80,9 +81,6 @@
     <t>Obligatorisk innlevering</t>
   </si>
   <si>
-    <t>01.10: **Oversiktsforelesning: Tidsrekker** i Aud A</t>
-  </si>
-  <si>
     <t xml:space="preserve">Regresjon </t>
   </si>
   <si>
@@ -98,9 +96,6 @@
     <t>Avansert regresjon og maskinlæring</t>
   </si>
   <si>
-    <t>10.09:  **Oppgaveseminar 2** i Aud A. Se \@ref(seminar) for oppgaver.</t>
-  </si>
-  <si>
     <t>21.09: **Oppgaveseminar 3** Aud A. Se \@ref(seminar) for oppgaver.</t>
   </si>
   <si>
@@ -113,12 +108,6 @@
     <t>03.09: (ingen aktivitet - se videoer og gjør oppgaver)</t>
   </si>
   <si>
-    <t>07.09:  (ingen aktivitet - jobb med dataøving 2)</t>
-  </si>
-  <si>
-    <t>28.09: (jobbe med obligatorisk innlevering)</t>
-  </si>
-  <si>
     <t>05.10: **Oversiktsforelesning: Tidsrekker** i Aud A</t>
   </si>
   <si>
@@ -140,54 +129,44 @@
     <t>12.11: (ingen aktivitet)</t>
   </si>
   <si>
-    <t>16:11: Kontakttime i Aud A</t>
-  </si>
-  <si>
-    <t>19:11: (ingen aktivitet)</t>
-  </si>
-  <si>
-    <t>02.11:  Praktisk informasjon om eksamen i Aud A</t>
-  </si>
-  <si>
-    <t>09.11:  Kontakttime i Aud A</t>
-  </si>
-  <si>
     <t>12.10: (ingen aktivitet - jobb med dataøving)</t>
   </si>
   <si>
-    <t xml:space="preserve">16.11: Kontakttime i Aud A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19.11: (ingen aktivitet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.08: **Introduksjon til MET4**. Aud A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07.09: (ingen aktivitet - jobb med dataøving 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.09: **Oppgaveseminar 2** i Aud A. Se \@ref(seminar) for oppgaver.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29.10: **Oppgaveseminar 6**, Aud A. Se \@ref(seminar) for oppgaver.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02.11: Praktisk informasjon om eksamen i Aud A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09.11: Kontakttime i Aud A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01.10: (ingen aktivitet - jobb med obligatorisk innlevering)</t>
+    <t>16.11: Kontakttime i Aud A</t>
+  </si>
+  <si>
+    <t>19.11: (ingen aktivitet)</t>
+  </si>
+  <si>
+    <t>17.08: **Introduksjon til MET4**. Aud A</t>
+  </si>
+  <si>
+    <t>07.09: (ingen aktivitet - jobb med dataøving 2)</t>
+  </si>
+  <si>
+    <t>10.09: **Oppgaveseminar 2** i Aud A. Se \@ref(seminar) for oppgaver.</t>
+  </si>
+  <si>
+    <t>29.10: **Oppgaveseminar 6**, Aud A. Se \@ref(seminar) for oppgaver.</t>
+  </si>
+  <si>
+    <t>02.11: Praktisk informasjon om eksamen i Aud A</t>
+  </si>
+  <si>
+    <t>09.11: Kontakttime i Aud A</t>
+  </si>
+  <si>
+    <t>01.10: (ingen aktivitet - jobb med obligatorisk innlevering)</t>
+  </si>
+  <si>
+    <t>28.09: (ingen aktivitet - jobb med obligatorisk innlevering)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -236,6 +215,7 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -523,16 +503,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="41.85546875" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="65.42578125" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="69.7109375" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="41.85546875" customWidth="1"/>
+    <col min="3" max="3" width="65.42578125" customWidth="1"/>
+    <col min="4" max="4" width="69.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -546,208 +526,208 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <v>35</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>36</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>37</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>38</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>39</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>37</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="D7" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>40</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>38</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="C8" s="1" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
         <v>41</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>42</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>42</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="D10" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
         <v>43</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
         <v>44</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
         <v>45</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
         <v>46</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
         <v>47</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
         <v>48</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>

</xml_diff>